<commit_message>
FIx formatting of letter decorators
</commit_message>
<xml_diff>
--- a/11-CollaborationList/CERN.xlsx
+++ b/11-CollaborationList/CERN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2050112399888/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2153813015232/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{8C08CD01-9107-394F-90A8-4EC6024BB625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6552E9C4-04B9-1D4F-9722-7F62A6ADC6F9}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{8C08CD01-9107-394F-90A8-4EC6024BB625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20F9044B-A97D-A646-BD86-F54122AC3763}"/>
   <bookViews>
-    <workbookView xWindow="10360" yWindow="4160" windowWidth="28040" windowHeight="17440" xr2:uid="{C85743D9-9737-224B-ABCC-C31CDEBE8F85}"/>
+    <workbookView xWindow="2200" yWindow="2200" windowWidth="28040" windowHeight="17440" xr2:uid="{C85743D9-9737-224B-ABCC-C31CDEBE8F85}"/>
   </bookViews>
   <sheets>
     <sheet name="CERN" sheetId="1" r:id="rId1"/>
@@ -85,13 +85,13 @@
     <t>CERN</t>
   </si>
   <si>
-    <t>CERN, CH-1211 Genève 23, Switzerland</t>
-  </si>
-  <si>
     <t>A.M Lombardi</t>
   </si>
   <si>
     <t>A.M.</t>
+  </si>
+  <si>
+    <t>CERN, CH-1211 Gen\`eve 23, Switzerland</t>
   </si>
 </sst>
 </file>
@@ -1070,19 +1070,19 @@
         <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
         <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>